<commit_message>
Update FPGA Excel spreadsheet
Replace binary Excel file in PCBNo.10081/FPGA (file changed: PCBNo.10081/FPGA/保正…?.xlsx). The diff is a binary change, so contents are not shown here — likely an update to FPGA-related data or BOM in the spreadsheet.
</commit_message>
<xml_diff>
--- a/PCBNo.10081/FPGA/修正履歴.xlsx
+++ b/PCBNo.10081/FPGA/修正履歴.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/512e22ffcc52695f/ドキュメント/GitHub/PCBNo.10081/PCBNo.10081/PCBNo.10081/SP0557_rev02_00_AI3/SP0557_rev02_00_AI3_2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/512e22ffcc52695f/ドキュメント/GitHub/PCBNo.10081/PCBNo.10081/FPGA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{BCDA7BAB-8026-4C53-BAA1-6CFCABC79B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41E34AB5-8F88-49EF-A593-73BDE1461DFE}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{BCDA7BAB-8026-4C53-BAA1-6CFCABC79B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74324252-AD45-4920-A6B2-E6EB76FC6AC7}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="7" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
+    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="2" activeTab="8" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
   </bookViews>
   <sheets>
     <sheet name="修正履歴" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="No5" sheetId="7" r:id="rId6"/>
     <sheet name="No6" sheetId="8" r:id="rId7"/>
     <sheet name="No.7" sheetId="9" r:id="rId8"/>
+    <sheet name="No.8" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="854" uniqueCount="752">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -5133,12 +5134,457 @@
   <si>
     <t>CLKCOM_OUT→CLK2（open接続のため不存在）、/CLK2A→.CLK2A（区切り文字統一）</t>
   </si>
+  <si>
+    <t>08</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自宅PCでワーニングが増える原因を解消</t>
+    <rPh sb="0" eb="2">
+      <t>ジタク</t>
+    </rPh>
+    <rPh sb="11" eb="12">
+      <t>フ</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>ゲンイン</t>
+    </rPh>
+    <rPh sb="17" eb="19">
+      <t>カイショウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Synplifyが自動でクロック制約を生成する設定になっている。自動生成の結果が間違っている。</t>
+  </si>
+  <si>
+    <t>実際の周期</t>
+  </si>
+  <si>
+    <t>自動生成の周期</t>
+  </si>
+  <si>
+    <t>倍率</t>
+  </si>
+  <si>
+    <t>CLKOS2 (20MHz)</t>
+  </si>
+  <si>
+    <t>50ns</t>
+  </si>
+  <si>
+    <t>6.2ns</t>
+  </si>
+  <si>
+    <t>8倍タイト</t>
+  </si>
+  <si>
+    <t>CLK20M (20MHz)</t>
+  </si>
+  <si>
+    <t>2.6ns</t>
+  </si>
+  <si>
+    <t>19倍タイト</t>
+  </si>
+  <si>
+    <t>CLKOS (100MHz)</t>
+  </si>
+  <si>
+    <t>10ns</t>
+  </si>
+  <si>
+    <t>4倍タイト</t>
+  </si>
+  <si>
+    <t>CLKOP (100MHz)</t>
+  </si>
+  <si>
+    <t>3.5ns</t>
+  </si>
+  <si>
+    <t>3倍タイト</t>
+  </si>
+  <si>
+    <t>CLKOS3 (10MHz)</t>
+  </si>
+  <si>
+    <t>100ns</t>
+  </si>
+  <si>
+    <t>定義漏れ</t>
+  </si>
+  <si>
+    <t>なぜ15,037件になるか</t>
+  </si>
+  <si>
+    <t>pll_gen.fdc が空 → SP0557.fdc のネット名が間違い（全無視）</t>
+  </si>
+  <si>
+    <t>→ frequency auto で AutoConstraint_SP0557.sdc を使用</t>
+  </si>
+  <si>
+    <t>→ 周期が3〜19倍タイト + 別clockgroup</t>
+  </si>
+  <si>
+    <t>→ 9,600個のFF × 6クロックドメインのほぼ全パスがタイミング違反</t>
+  </si>
+  <si>
+    <t>→ 各違反パスにワーニング出力 → 15,037件</t>
+  </si>
+  <si>
+    <t>なぜ職場PCでは16件だったか</t>
+  </si>
+  <si>
+    <r>
+      <t>1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>SP0557_syn.prj</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>frequency auto</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (自動制約モード)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>AutoConstraint_SP0557.sdc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: クロック周期が大幅に間違い</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>さらに各クロックが</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>別々のclockgroup</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>に配置 → クロスドメイン解析が不正確</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>SP0557.fdc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: ネット名が間違い → Synplifyが全制約をサイレントに無視</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>{n:slv_com_top_inst.clk_gen_inst2.PLL_inst.CLKCOM_OUT}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> 等の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>存在しないネット名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>で参照しているため、正しい制約が書かれていても全て無視される。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>pll_gen.fdc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 空ファイル（IPコアのスタブのみ）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>職場PCは </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>C:\work\S127M\PCBNo_10081\SP0557_rev02_00_AI3\</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> でgitとは</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>別の独立コピー</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>。そちらでは</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>.prj</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>や制約ファイルが正しく設定されていた（手動修正またはSynplifyキャッシュによる）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>既にコミット </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>22fa5be</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> で修正済み（このブランチに含まれている）:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>frequency auto</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>100.0</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>pll_gen.fdc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> に正しいPLLポート名 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>{p:CLKOP}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> 等でクロック定義追加</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SP0557.fdc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> を pll_gen.fdc のクロック名を参照する形にリライト</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>AutoConstraint_SP0557.sdc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> を無効化</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>家PCでの復旧手順</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: このブランチをmasterにマージ → Diamond でClean → Synthesize Design → 16件に戻るはず。</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="27">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5333,6 +5779,24 @@
       <family val="3"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="13.5"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -5398,7 +5862,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -5643,6 +6107,24 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6092,9 +6574,15 @@
       <c r="F11" s="26"/>
     </row>
     <row r="12" spans="3:6">
-      <c r="C12" s="26"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="27"/>
+      <c r="C12" s="26">
+        <v>8</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>710</v>
+      </c>
+      <c r="E12" s="27" t="s">
+        <v>711</v>
+      </c>
       <c r="F12" s="26"/>
     </row>
     <row r="13" spans="3:6">
@@ -10263,4 +10751,219 @@
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1C504B7-EEB2-42BE-916D-0045C563FE42}">
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="70.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18.75">
+      <c r="A1" s="82" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="9" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18.75">
+      <c r="A3" s="82" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="31.5">
+      <c r="A4" s="83" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="83" t="s">
+        <v>713</v>
+      </c>
+      <c r="C4" s="83" t="s">
+        <v>714</v>
+      </c>
+      <c r="D4" s="84" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" thickBot="1">
+      <c r="A5" s="7" t="s">
+        <v>716</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>717</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>718</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="32.25" thickBot="1">
+      <c r="A6" s="7" t="s">
+        <v>720</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>717</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>721</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" thickBot="1">
+      <c r="A7" s="7" t="s">
+        <v>723</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>721</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" thickBot="1">
+      <c r="A8" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="7" t="s">
+        <v>729</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>730</v>
+      </c>
+      <c r="C9" s="85" t="s">
+        <v>731</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="9" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="18.75">
+      <c r="A11" s="82" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="31.5">
+      <c r="A12" s="21" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="18.75">
+      <c r="A13" s="82" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="18.75">
+      <c r="A15" s="82" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="1" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="1" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="1" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="1" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="1" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="18.75">
+      <c r="A21" s="82" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="47.25">
+      <c r="A22" s="9" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="18.75">
+      <c r="A23" s="82" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="9" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="11"/>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="86" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="86" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="86" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="86" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="31.5">
+      <c r="A31" s="87" t="s">
+        <v>751</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update FPGA Excel file
Updated binary Excel workbook in PCBNo.10081/FPGA. The file contents differ (binary change); no textual diff is available. This likely contains updated FPGA-related spreadsheet data (e.g., BOM or configuration) for PCB No.10081.
</commit_message>
<xml_diff>
--- a/PCBNo.10081/FPGA/修正履歴.xlsx
+++ b/PCBNo.10081/FPGA/修正履歴.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/512e22ffcc52695f/ドキュメント/GitHub/PCBNo.10081/PCBNo.10081/FPGA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{BCDA7BAB-8026-4C53-BAA1-6CFCABC79B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74324252-AD45-4920-A6B2-E6EB76FC6AC7}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{BCDA7BAB-8026-4C53-BAA1-6CFCABC79B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9DB8534-7D9A-49AF-85EB-704BE2F56C5F}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="2" activeTab="8" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="9" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
   </bookViews>
   <sheets>
     <sheet name="修正履歴" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="No6" sheetId="8" r:id="rId7"/>
     <sheet name="No.7" sheetId="9" r:id="rId8"/>
     <sheet name="No.8" sheetId="10" r:id="rId9"/>
+    <sheet name="No.9" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="854" uniqueCount="752">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="836">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -5577,6 +5578,657 @@
         <charset val="128"/>
       </rPr>
       <t>: このブランチをmasterにマージ → Diamond でClean → Synthesize Design → 16件に戻るはず。</t>
+    </r>
+  </si>
+  <si>
+    <t>09_1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>No1~8が適応できているかの確認</t>
+    <rPh sb="6" eb="8">
+      <t>テキオウ</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>修正履歴No.1〜No.8の適用確認を行った結果、コードレベルでは全修正が適用済みだが、コンパイル結果に以下4つの残存問題がある。本計画でこれら全てを修正する。</t>
+  </si>
+  <si>
+    <t>修正1: CD134 識別子エラー修正（3件）</t>
+  </si>
+  <si>
+    <t>原因</t>
+  </si>
+  <si>
+    <t>変更前:</t>
+  </si>
+  <si>
+    <t>変更後:</t>
+  </si>
+  <si>
+    <t>-- ENB_START preservation handled by SP0557.fdc (Section 7N)</t>
+  </si>
+  <si>
+    <t>-- DATAOUT preservation handled by SP0557.fdc (Section 7E)</t>
+  </si>
+  <si>
+    <t>-- NODE preservation handled by SP0557.fdc (Section 7D)</t>
+  </si>
+  <si>
+    <t>### 原因</t>
+  </si>
+  <si>
+    <t>### 修正内容</t>
+  </si>
+  <si>
+    <t>修正4: SLICE使用率改善</t>
+  </si>
+  <si>
+    <t>対応方針</t>
+  </si>
+  <si>
+    <t>修正3の115MHz→100MHz変更により、以下の改善が期待される:</t>
+  </si>
+  <si>
+    <t>Synplifyのレジスタ複製削減（タイミング圧力緩和）</t>
+  </si>
+  <si>
+    <t>P&amp;Rの配置最適化余地拡大</t>
+  </si>
+  <si>
+    <t>推定効果: 89% → 85-87%程度</t>
+  </si>
+  <si>
+    <t>追加のRTL変更は行わない（修正2のFDCクロック定義が正しく適用されれば、合成最適化の質も改善される）。</t>
+  </si>
+  <si>
+    <t>修正対象ファイル一覧</t>
+  </si>
+  <si>
+    <t>RTL/SP0557/compactppmc/ppmc_ctrl.vhd</t>
+  </si>
+  <si>
+    <t>ENB_START属性削除</t>
+  </si>
+  <si>
+    <t>RTL/SP0557/slv_com/rx_com/dec6b_5b.vhd</t>
+  </si>
+  <si>
+    <t>DATAOUT属性削除</t>
+  </si>
+  <si>
+    <t>RTL/SP0557/slv_com/slv_ctrl/slv_rx_ctrl.vhd</t>
+  </si>
+  <si>
+    <t>NODE属性削除</t>
+  </si>
+  <si>
+    <t>RTL/IPcore/pll_gen/pll_gen.fdc</t>
+  </si>
+  <si>
+    <t>FPGA/SP0557.lpf</t>
+  </si>
+  <si>
+    <t>115MHz → 100MHz</t>
+  </si>
+  <si>
+    <t>修正適用後、Lattice Diamond / Synplifyでフルビルドを実施し、以下を確認:</t>
+  </si>
+  <si>
+    <t>BN137, MO160, MO129, CL177, CL240, CD638 が消滅したままであること</t>
+  </si>
+  <si>
+    <t>全クロックドメインの制約がPASSすること（CLKCOM_OUT含む）</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">RTLソースファイル内で </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>attribute syn_preserve of XXXX : signal is true;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> と記述しているが、対象がエンティティの</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>出力ポート</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>であるため、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: signal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> ではなく </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: port</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> を使う必要がある。FDCファイル(SP0557.fdc)には既に正しい制約が定義されているため、RTL内の重複属性を削除するのが最もクリーン。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ファイル1: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>PCBNo.10081/FPGA/RTL/SP0557/compactppmc/ppmc_ctrl.vhd</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (133-136行)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">削除: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ENB_START</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> のsyn_preserve属性宣言（ENB_STARTは出力ポート）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>s_pls_ld</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> は内部signal なので残す</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SP0557.fdc 7N節（246行: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>define_attribute {v:work.ppmc_ctrl} syn_preserve {1}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>）がモジュール全体を保護しているため、RTL属性は不要</t>
+    </r>
+  </si>
+  <si>
+    <t>attribute syn_preserve : boolean;</t>
+  </si>
+  <si>
+    <t>attribute syn_preserve of s_pls_ld  : signal is true;</t>
+  </si>
+  <si>
+    <t>attribute syn_preserve of ENB_START : signal is true;</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ファイル2: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>PCBNo.10081/FPGA/RTL/SP0557/slv_com/rx_com/dec6b_5b.vhd</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (36-38行)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">削除: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>DATAOUT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> のsyn_preserve属性宣言（DATAOUTは出力ポート）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SP0557.fdc 7E節（166-171行）が合成後レジスタ名 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>DATAOUT_33_0_areg[*]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> で保護済み</t>
+    </r>
+  </si>
+  <si>
+    <t>attribute syn_preserve of DATAOUT : signal is true;</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ファイル3: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>PCBNo.10081/FPGA/RTL/SP0557/slv_com/slv_ctrl/slv_rx_ctrl.vhd</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (90-94行)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">削除: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>NODE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> のsyn_preserve属性宣言（NODEは出力ポート）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>byte_cnt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> はinternal signal なので残す</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SP0557.fdc 7D節（159-162行）が </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>NODE[0:3]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> を階層パス付きで保護済み</t>
+    </r>
+  </si>
+  <si>
+    <t>attribute syn_keep : boolean;</t>
+  </si>
+  <si>
+    <t>attribute syn_keep of byte_cnt : signal is true;</t>
+  </si>
+  <si>
+    <t>attribute syn_preserve of NODE : signal is true;</t>
+  </si>
+  <si>
+    <t>## 修正2: MT420/MT529 警告修正（10件）</t>
+  </si>
+  <si>
+    <t>`pll_gen.fdc` で `{p:CLKOP}` 等のポート参照構文を使用しているが、Synplifyは内部信号 `CLKOP_t` からクロックを推論し、`pll_gen|CLKOP_inferred_clock` という名前を生成する。FDCのポート参照と推論クロック名が一致しないため、FDCのdefine_clockが**黙殺**されている。</t>
+  </si>
+  <si>
+    <t>結果として全PLLクロックが `set_option -frequency 100.0` の10ns周期（100MHz）で処理され、実際の周波数と一致しないクロック（CLKOS2=20MHz, CLKOS3=10MHz）で不正確な合成最適化が行われている。</t>
+  </si>
+  <si>
+    <t>**ファイル: `PCBNo.10081/FPGA/RTL/IPcore/pll_gen/pll_gen.fdc`**</t>
+  </si>
+  <si>
+    <t>`{p:PORT}` 構文を `{n:SIGNAL}` 構文に変更し、Synplifyが実際に推論する内部信号名を参照する。</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOP_100M} {p:CLKOP} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS_100M_90} {p:CLKOS} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS2_20M} {p:CLKOS2} -freq 20.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS3_10M} {p:CLKOS3} -freq 10.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOP_100M} {n:CLKOP_t} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS_100M_90} {n:CLKOS_t} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS2_20M} {n:CLKOS2_t} -freq 20.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS3_10M} {n:CLKOS3_t} -freq 10.000 ...</t>
+  </si>
+  <si>
+    <t>`CLKOP_t`, `CLKOS_t`, `CLKOS2_t`, `CLKOS3_t` は `pll_gen.vhd` の23-30行で宣言された内部信号で、EHXPLLLプリミティブの出力に直接接続されている（79-80行）。</t>
+  </si>
+  <si>
+    <t>**注意**: `{n:SIGNAL}` が効かない場合のフォールバックとして、EHXPLLLインスタンスの出力ピンを直接参照する構文も検討:</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOP_100M} {n:PLLInst_0.CLKOP} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>## 修正3: CLKCOM_OUT タイミング違反修正</t>
+  </si>
+  <si>
+    <t>LPFで100MHzクロックに115MHzのガードバンド制約を設定しているが、DCFIFO Block RAM出力→TX制御レジスタのクリティカルパスが9.823ns（C2Q: 5.830ns + routing: 2.874ns + LUT: 0.236ns）で、8.696ns（115MHz）の制約を1.275ns超過している。</t>
+  </si>
+  <si>
+    <t>100MHz（10ns周期）なら9.852nsの余裕があり、マージナルだがPASSする。</t>
+  </si>
+  <si>
+    <t>**ファイル: `PCBNo.10081/FPGA/SP0557.lpf` (303-304行)**</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET "slv_com_top_inst.CLK2" 115.000000 MHz ;</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET "slv_com_top_inst.CLK2A" 115.000000 MHz ;</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET "slv_com_top_inst.CLK2" 100.000000 MHz ;</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET "slv_com_top_inst.CLK2A" 100.000000 MHz ;</t>
+  </si>
+  <si>
+    <r>
+      <t>LPFコメント更新</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: Section 1のガードバンドに関するコメント（299行）を更新し、115MHz→100MHzに戻した理由を記載</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>{p:PORT}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>{n:SIGNAL_t}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1. CD134エラー</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 3件 → 0件になること</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. MT420/MT529警告</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 10件 → 0件（または大幅減少）になること</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>{n:SIGNAL_t}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> が効かない場合は代替構文を試行</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3. CLKCOM_OUT制約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 100MHz制約でsetup/hold共にPASSすること</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. Hold違反</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 4件 → 0件になること（115MHz緩和による改善）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5. SLICE使用率</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 89%から低下していること</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>6. 既存の修正が壊れていないこと</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>:</t>
     </r>
   </si>
 </sst>
@@ -5786,13 +6438,14 @@
       <charset val="128"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <name val="Meiryo UI"/>
       <family val="3"/>
       <charset val="128"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="10"/>
       <name val="Meiryo UI"/>
       <family val="3"/>
       <charset val="128"/>
@@ -5862,7 +6515,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6112,20 +6765,23 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6586,9 +7242,15 @@
       <c r="F12" s="26"/>
     </row>
     <row r="13" spans="3:6">
-      <c r="C13" s="26"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="27"/>
+      <c r="C13" s="26">
+        <v>9</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>752</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>753</v>
+      </c>
       <c r="F13" s="26"/>
     </row>
     <row r="14" spans="3:6">
@@ -6704,6 +7366,628 @@
       <c r="D32" s="29"/>
       <c r="E32" s="27"/>
       <c r="F32" s="26"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14089E9A-DD6C-474E-BC76-1DCDCF7A2A9D}">
+  <dimension ref="A1:B181"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="24">
+      <c r="A1" s="14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="1" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="24">
+      <c r="A7" s="14" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="18.75">
+      <c r="A9" s="15" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="1" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="18.75">
+      <c r="A13" s="15" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="17" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="18"/>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="18" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="24" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="18" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="1" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="16" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="16" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="1" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" s="16" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" s="16" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" s="17" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="18"/>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="18" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" s="18" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="1" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" s="16" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" s="1" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" s="16" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="17" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" s="18"/>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" s="18" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" s="24" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" s="18" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="1" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="16" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="16" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" s="16" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" s="1" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" s="16" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="16" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" s="16" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" s="16" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" s="16" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" s="16" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="16" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" s="16" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" s="16" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" s="16" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" s="16" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" s="16" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" s="16" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" s="16" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" s="16" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" s="16" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" s="16" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" s="16" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="16" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" s="16" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" s="16" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" s="16" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" s="16" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" s="16" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" s="16" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" s="16" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" s="16" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" s="16" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" s="16" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" s="16" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128" s="16" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" s="16" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" s="16" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133" s="16" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1">
+      <c r="A136" s="16" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1">
+      <c r="A137" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138" s="16" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1">
+      <c r="A139" s="16" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1">
+      <c r="A141" s="17" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" ht="24">
+      <c r="A145" s="14" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" ht="18.75">
+      <c r="A147" s="15" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" s="1" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" s="18"/>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" s="18" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" s="18" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" s="18" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" s="1" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" ht="24">
+      <c r="A159" s="14" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B161" s="20" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" ht="71.25">
+      <c r="A162" s="21" t="s">
+        <v>772</v>
+      </c>
+      <c r="B162" s="9" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" ht="71.25">
+      <c r="A163" s="21" t="s">
+        <v>774</v>
+      </c>
+      <c r="B163" s="9" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" ht="71.25">
+      <c r="A164" s="21" t="s">
+        <v>776</v>
+      </c>
+      <c r="B164" s="9" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" ht="60">
+      <c r="A165" s="21" t="s">
+        <v>778</v>
+      </c>
+      <c r="B165" s="21" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" ht="47.25">
+      <c r="A166" s="21" t="s">
+        <v>779</v>
+      </c>
+      <c r="B166" s="9" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" ht="24">
+      <c r="A169" s="14" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="1" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="18"/>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="19" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="19" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="88" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="19" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1">
+      <c r="A177" s="19" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1">
+      <c r="A178" s="19" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1">
+      <c r="A179" s="19" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1">
+      <c r="A180" s="25" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1">
+      <c r="A181" s="25" t="s">
+        <v>783</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>

</xml_diff>

<commit_message>
Update FPGA Excel file for PCBNo.10081
Replace the binary .xlsx spreadsheet in PCBNo.10081/FPGA. The Excel file has been updated (binary changes) to reflect revisions in the FPGA documentation/data.
</commit_message>
<xml_diff>
--- a/PCBNo.10081/FPGA/修正履歴.xlsx
+++ b/PCBNo.10081/FPGA/修正履歴.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/512e22ffcc52695f/ドキュメント/GitHub/PCBNo.10081/PCBNo.10081/FPGA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FPGA work\PCBNo.10081\FPGA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{BCDA7BAB-8026-4C53-BAA1-6CFCABC79B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74324252-AD45-4920-A6B2-E6EB76FC6AC7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F38BC98-97EE-4E89-B636-CBEA2B7A2410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="2" activeTab="8" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
   </bookViews>
   <sheets>
     <sheet name="修正履歴" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,9 @@
     <sheet name="No6" sheetId="8" r:id="rId7"/>
     <sheet name="No.7" sheetId="9" r:id="rId8"/>
     <sheet name="No.8" sheetId="10" r:id="rId9"/>
+    <sheet name="No.9" sheetId="11" r:id="rId10"/>
+    <sheet name="No.10" sheetId="12" r:id="rId11"/>
+    <sheet name="No.11" sheetId="13" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="854" uniqueCount="752">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="1021">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -5579,12 +5582,1654 @@
       <t>: このブランチをmasterにマージ → Diamond でClean → Synthesize Design → 16件に戻るはず。</t>
     </r>
   </si>
+  <si>
+    <t>09_1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>No1~8が適応できているかの確認</t>
+    <rPh sb="6" eb="8">
+      <t>テキオウ</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>修正履歴No.1〜No.8の適用確認を行った結果、コードレベルでは全修正が適用済みだが、コンパイル結果に以下4つの残存問題がある。本計画でこれら全てを修正する。</t>
+  </si>
+  <si>
+    <t>修正1: CD134 識別子エラー修正（3件）</t>
+  </si>
+  <si>
+    <t>原因</t>
+  </si>
+  <si>
+    <t>変更前:</t>
+  </si>
+  <si>
+    <t>変更後:</t>
+  </si>
+  <si>
+    <t>-- ENB_START preservation handled by SP0557.fdc (Section 7N)</t>
+  </si>
+  <si>
+    <t>-- DATAOUT preservation handled by SP0557.fdc (Section 7E)</t>
+  </si>
+  <si>
+    <t>-- NODE preservation handled by SP0557.fdc (Section 7D)</t>
+  </si>
+  <si>
+    <t>### 原因</t>
+  </si>
+  <si>
+    <t>### 修正内容</t>
+  </si>
+  <si>
+    <t>修正4: SLICE使用率改善</t>
+  </si>
+  <si>
+    <t>対応方針</t>
+  </si>
+  <si>
+    <t>修正3の115MHz→100MHz変更により、以下の改善が期待される:</t>
+  </si>
+  <si>
+    <t>Synplifyのレジスタ複製削減（タイミング圧力緩和）</t>
+  </si>
+  <si>
+    <t>P&amp;Rの配置最適化余地拡大</t>
+  </si>
+  <si>
+    <t>推定効果: 89% → 85-87%程度</t>
+  </si>
+  <si>
+    <t>追加のRTL変更は行わない（修正2のFDCクロック定義が正しく適用されれば、合成最適化の質も改善される）。</t>
+  </si>
+  <si>
+    <t>修正対象ファイル一覧</t>
+  </si>
+  <si>
+    <t>RTL/SP0557/compactppmc/ppmc_ctrl.vhd</t>
+  </si>
+  <si>
+    <t>ENB_START属性削除</t>
+  </si>
+  <si>
+    <t>RTL/SP0557/slv_com/rx_com/dec6b_5b.vhd</t>
+  </si>
+  <si>
+    <t>DATAOUT属性削除</t>
+  </si>
+  <si>
+    <t>RTL/SP0557/slv_com/slv_ctrl/slv_rx_ctrl.vhd</t>
+  </si>
+  <si>
+    <t>NODE属性削除</t>
+  </si>
+  <si>
+    <t>RTL/IPcore/pll_gen/pll_gen.fdc</t>
+  </si>
+  <si>
+    <t>FPGA/SP0557.lpf</t>
+  </si>
+  <si>
+    <t>115MHz → 100MHz</t>
+  </si>
+  <si>
+    <t>修正適用後、Lattice Diamond / Synplifyでフルビルドを実施し、以下を確認:</t>
+  </si>
+  <si>
+    <t>BN137, MO160, MO129, CL177, CL240, CD638 が消滅したままであること</t>
+  </si>
+  <si>
+    <t>全クロックドメインの制約がPASSすること（CLKCOM_OUT含む）</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">RTLソースファイル内で </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>attribute syn_preserve of XXXX : signal is true;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> と記述しているが、対象がエンティティの</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>出力ポート</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>であるため、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: signal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> ではなく </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: port</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> を使う必要がある。FDCファイル(SP0557.fdc)には既に正しい制約が定義されているため、RTL内の重複属性を削除するのが最もクリーン。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ファイル1: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>PCBNo.10081/FPGA/RTL/SP0557/compactppmc/ppmc_ctrl.vhd</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (133-136行)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">削除: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ENB_START</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> のsyn_preserve属性宣言（ENB_STARTは出力ポート）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>s_pls_ld</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> は内部signal なので残す</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SP0557.fdc 7N節（246行: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>define_attribute {v:work.ppmc_ctrl} syn_preserve {1}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>）がモジュール全体を保護しているため、RTL属性は不要</t>
+    </r>
+  </si>
+  <si>
+    <t>attribute syn_preserve : boolean;</t>
+  </si>
+  <si>
+    <t>attribute syn_preserve of s_pls_ld  : signal is true;</t>
+  </si>
+  <si>
+    <t>attribute syn_preserve of ENB_START : signal is true;</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ファイル2: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>PCBNo.10081/FPGA/RTL/SP0557/slv_com/rx_com/dec6b_5b.vhd</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (36-38行)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">削除: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>DATAOUT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> のsyn_preserve属性宣言（DATAOUTは出力ポート）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SP0557.fdc 7E節（166-171行）が合成後レジスタ名 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>DATAOUT_33_0_areg[*]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> で保護済み</t>
+    </r>
+  </si>
+  <si>
+    <t>attribute syn_preserve of DATAOUT : signal is true;</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ファイル3: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>PCBNo.10081/FPGA/RTL/SP0557/slv_com/slv_ctrl/slv_rx_ctrl.vhd</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> (90-94行)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">削除: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>NODE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> のsyn_preserve属性宣言（NODEは出力ポート）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>byte_cnt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> はinternal signal なので残す</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SP0557.fdc 7D節（159-162行）が </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>NODE[0:3]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> を階層パス付きで保護済み</t>
+    </r>
+  </si>
+  <si>
+    <t>attribute syn_keep : boolean;</t>
+  </si>
+  <si>
+    <t>attribute syn_keep of byte_cnt : signal is true;</t>
+  </si>
+  <si>
+    <t>attribute syn_preserve of NODE : signal is true;</t>
+  </si>
+  <si>
+    <t>## 修正2: MT420/MT529 警告修正（10件）</t>
+  </si>
+  <si>
+    <t>`pll_gen.fdc` で `{p:CLKOP}` 等のポート参照構文を使用しているが、Synplifyは内部信号 `CLKOP_t` からクロックを推論し、`pll_gen|CLKOP_inferred_clock` という名前を生成する。FDCのポート参照と推論クロック名が一致しないため、FDCのdefine_clockが**黙殺**されている。</t>
+  </si>
+  <si>
+    <t>結果として全PLLクロックが `set_option -frequency 100.0` の10ns周期（100MHz）で処理され、実際の周波数と一致しないクロック（CLKOS2=20MHz, CLKOS3=10MHz）で不正確な合成最適化が行われている。</t>
+  </si>
+  <si>
+    <t>**ファイル: `PCBNo.10081/FPGA/RTL/IPcore/pll_gen/pll_gen.fdc`**</t>
+  </si>
+  <si>
+    <t>`{p:PORT}` 構文を `{n:SIGNAL}` 構文に変更し、Synplifyが実際に推論する内部信号名を参照する。</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOP_100M} {p:CLKOP} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS_100M_90} {p:CLKOS} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS2_20M} {p:CLKOS2} -freq 20.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS3_10M} {p:CLKOS3} -freq 10.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOP_100M} {n:CLKOP_t} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS_100M_90} {n:CLKOS_t} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS2_20M} {n:CLKOS2_t} -freq 20.000 ...</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOS3_10M} {n:CLKOS3_t} -freq 10.000 ...</t>
+  </si>
+  <si>
+    <t>`CLKOP_t`, `CLKOS_t`, `CLKOS2_t`, `CLKOS3_t` は `pll_gen.vhd` の23-30行で宣言された内部信号で、EHXPLLLプリミティブの出力に直接接続されている（79-80行）。</t>
+  </si>
+  <si>
+    <t>**注意**: `{n:SIGNAL}` が効かない場合のフォールバックとして、EHXPLLLインスタンスの出力ピンを直接参照する構文も検討:</t>
+  </si>
+  <si>
+    <t>define_clock -name {CLKOP_100M} {n:PLLInst_0.CLKOP} -freq 100.000 ...</t>
+  </si>
+  <si>
+    <t>## 修正3: CLKCOM_OUT タイミング違反修正</t>
+  </si>
+  <si>
+    <t>LPFで100MHzクロックに115MHzのガードバンド制約を設定しているが、DCFIFO Block RAM出力→TX制御レジスタのクリティカルパスが9.823ns（C2Q: 5.830ns + routing: 2.874ns + LUT: 0.236ns）で、8.696ns（115MHz）の制約を1.275ns超過している。</t>
+  </si>
+  <si>
+    <t>100MHz（10ns周期）なら9.852nsの余裕があり、マージナルだがPASSする。</t>
+  </si>
+  <si>
+    <t>**ファイル: `PCBNo.10081/FPGA/SP0557.lpf` (303-304行)**</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET "slv_com_top_inst.CLK2" 115.000000 MHz ;</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET "slv_com_top_inst.CLK2A" 115.000000 MHz ;</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET "slv_com_top_inst.CLK2" 100.000000 MHz ;</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET "slv_com_top_inst.CLK2A" 100.000000 MHz ;</t>
+  </si>
+  <si>
+    <r>
+      <t>LPFコメント更新</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: Section 1のガードバンドに関するコメント（299行）を更新し、115MHz→100MHzに戻した理由を記載</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>{p:PORT}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>{n:SIGNAL_t}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1. CD134エラー</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 3件 → 0件になること</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. MT420/MT529警告</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 10件 → 0件（または大幅減少）になること</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>{n:SIGNAL_t}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve"> が効かない場合は代替構文を試行</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3. CLKCOM_OUT制約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 100MHz制約でsetup/hold共にPASSすること</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. Hold違反</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 4件 → 0件になること（115MHz緩和による改善）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5. SLICE使用率</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: 89%から低下していること</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>6. 既存の修正が壊れていないこと</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>:</t>
+    </r>
+  </si>
+  <si>
+    <t>10</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>No1~9の確認</t>
+    <rPh sb="6" eb="8">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>FDCファイルがDiamondプロジェクトに未登録</t>
+  </si>
+  <si>
+    <t>修正履歴 No.1〜9 コンパイル結果検証レポート</t>
+  </si>
+  <si>
+    <t>コンパイル日時: 2026-02-28 (SP0557_SP0557.srr / SP0557_SP0557.twr)</t>
+  </si>
+  <si>
+    <t>全体結果サマリ</t>
+  </si>
+  <si>
+    <t>区分</t>
+  </si>
+  <si>
+    <t>コンパイルエラー</t>
+  </si>
+  <si>
+    <t>Setupタイミング違反</t>
+  </si>
+  <si>
+    <t>Holdタイミング違反</t>
+  </si>
+  <si>
+    <t>合成ワーニング</t>
+  </si>
+  <si>
+    <t>272件</t>
+  </si>
+  <si>
+    <t>修正No.9で計画した4つの修正の適用状況</t>
+  </si>
+  <si>
+    <t>修正1: CD134 識別子エラー修正（3件） → 適用済み・効果あり</t>
+  </si>
+  <si>
+    <t>ソース状態</t>
+  </si>
+  <si>
+    <t>コンパイル反映</t>
+  </si>
+  <si>
+    <t>ppmc_ctrl.vhd:133-136</t>
+  </si>
+  <si>
+    <t>ENB_START syn_preserve削除</t>
+  </si>
+  <si>
+    <t>適用済み</t>
+  </si>
+  <si>
+    <t>dec6b_5b.vhd:36-37</t>
+  </si>
+  <si>
+    <t>DATAOUT syn_preserve削除</t>
+  </si>
+  <si>
+    <t>slv_rx_ctrl.vhd:90-93</t>
+  </si>
+  <si>
+    <t>NODE syn_preserve削除</t>
+  </si>
+  <si>
+    <t>s_pls_ld / byte_cnt の属性も正しく保持されています。</t>
+  </si>
+  <si>
+    <t>修正2: MT420/MT529 PLL クロック制約修正 → ソース適用済みだがコンパイル未反映（致命的）</t>
+  </si>
+  <si>
+    <t>問題: FDCファイルがSynplifyに読み込まれていない</t>
+  </si>
+  <si>
+    <t>合成レポート 1240行目:</t>
+  </si>
+  <si>
+    <t>@A: MF827 |No constraint file specified.</t>
+  </si>
+  <si>
+    <t>Removed file: C:\FPGA work\PCBNo.10081\FPGA\RTL\IPcore\pll_gen\pll_gen.fdc</t>
+  </si>
+  <si>
+    <t>Removed file: C:\FPGA work\PCBNo.10081\FPGA\SP0557\SP0557.fdc</t>
+  </si>
+  <si>
+    <t>@W: MT420 |Found inferred clock pll_gen|CLKOS2_inferred_clock with period 5.00ns</t>
+  </si>
+  <si>
+    <t>@W: MT420 |Found inferred clock SP0557|CLK20M with period 5.00ns</t>
+  </si>
+  <si>
+    <t>@W: MT420 |Found inferred clock pll_gen|CLKOS_inferred_clock with period 5.00ns</t>
+  </si>
+  <si>
+    <t>@W: MT420 |Found inferred clock pll_gen|CLKOP_inferred_clock with period 5.00ns</t>
+  </si>
+  <si>
+    <t>@W: MT420 |Found inferred clock pll_gen|CLKOS3_inferred_clock with period 5.00ns</t>
+  </si>
+  <si>
+    <t>全PLLクロックがデフォルト200MHz (5ns)として推定され、FDCのclock group/multicycle/false path制約も全て無効です。</t>
+  </si>
+  <si>
+    <t>修正3: CLKCOM_OUT タイミング違反修正 → 一部適用だが主要制約が未反映（致命的）</t>
+  </si>
+  <si>
+    <t>UP_TXD SLEWRATE=FAST</t>
+  </si>
+  <si>
+    <t>FREQUENCY PORT "UP_CLK" 20MHz</t>
+  </si>
+  <si>
+    <t>FREQUENCY NET制約 (5クロック)</t>
+  </si>
+  <si>
+    <t>適用済み・反映あり</t>
+  </si>
+  <si>
+    <t>BLOCK PATH CLK20M_c &lt;-&gt; s_PLL_CLK20M/CLK1</t>
+  </si>
+  <si>
+    <t>MULTICYCLE s_PLL_CLK20M &lt;-&gt; CLK1 (2X)</t>
+  </si>
+  <si>
+    <t>問題: LPFのクロックネット名が実際のPAR認識名と不一致</t>
+  </si>
+  <si>
+    <t>LPF記述</t>
+  </si>
+  <si>
+    <t>PARが認識する実際のネット名</t>
+  </si>
+  <si>
+    <t>slv_com_top_inst.CLK2</t>
+  </si>
+  <si>
+    <t>slv_com_top_inst.CLKCOM_OUT</t>
+  </si>
+  <si>
+    <t>不一致</t>
+  </si>
+  <si>
+    <t>slv_com_top_inst.CLK2A</t>
+  </si>
+  <si>
+    <t>LPF Section</t>
+  </si>
+  <si>
+    <t>制約</t>
+  </si>
+  <si>
+    <t>影響</t>
+  </si>
+  <si>
+    <t>Section 2 (一部)</t>
+  </si>
+  <si>
+    <t>BLOCK PATH CLK20M_c &lt;-&gt; CLK2/CLK2A</t>
+  </si>
+  <si>
+    <t>CLK20M_c→CLKCOM_OUT/CLK2Aパスが解析対象に残存</t>
+  </si>
+  <si>
+    <t>Section 4</t>
+  </si>
+  <si>
+    <t>BLOCK PATH s_PLL_CLK20M &lt;-&gt; CLK2/CLK2A</t>
+  </si>
+  <si>
+    <t>20MHz↔100MHzパスが未遮断</t>
+  </si>
+  <si>
+    <t>Section 5</t>
+  </si>
+  <si>
+    <t>MULTICYCLE CLK1 &lt;-&gt; CLK2 (10X/2X)</t>
+  </si>
+  <si>
+    <t>59パスが100MHz解析下に残存（最大の問題）</t>
+  </si>
+  <si>
+    <t>Section 6</t>
+  </si>
+  <si>
+    <t>MULTICYCLE CLK1 &lt;-&gt; CLK2A (10X/2X)</t>
+  </si>
+  <si>
+    <t>CLK1↔CLK2Aパスが緩和されず</t>
+  </si>
+  <si>
+    <t>TWR（タイミングレポート）で確認した証拠:</t>
+  </si>
+  <si>
+    <t>タイミング結果詳細 (TWR)</t>
+  </si>
+  <si>
+    <t>クロックドメイン</t>
+  </si>
+  <si>
+    <t>実測</t>
+  </si>
+  <si>
+    <t>スラック</t>
+  </si>
+  <si>
+    <t>100.000 MHz</t>
+  </si>
+  <si>
+    <t>98.483 MHz</t>
+  </si>
+  <si>
+    <t>-0.154ns</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>CLK2A (100MHz)</t>
+  </si>
+  <si>
+    <t>271.370 MHz</t>
+  </si>
+  <si>
+    <t>+6.315ns</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>20.000 MHz</t>
+  </si>
+  <si>
+    <t>67.645 MHz</t>
+  </si>
+  <si>
+    <t>充分</t>
+  </si>
+  <si>
+    <t>CLK1 (10MHz)</t>
+  </si>
+  <si>
+    <t>10.000 MHz</t>
+  </si>
+  <si>
+    <t>14.067 MHz</t>
+  </si>
+  <si>
+    <t>UP_CLK_c (20MHz)</t>
+  </si>
+  <si>
+    <t>(パスなし)</t>
+  </si>
+  <si>
+    <t>必要な修正アクション</t>
+  </si>
+  <si>
+    <t>アクション1 (最優先): SP0557.ldfにFDCファイルを登録</t>
+  </si>
+  <si>
+    <t>これにより:</t>
+  </si>
+  <si>
+    <t>MT420/MT529ワーニングが解消</t>
+  </si>
+  <si>
+    <t>PLLクロックが正しい周波数で合成最適化される</t>
+  </si>
+  <si>
+    <t>FDCのmulticycle/false path制約がSynplify合成時に有効化される</t>
+  </si>
+  <si>
+    <t>アクション2 (最優先): LPFクロックネット名の修正</t>
+  </si>
+  <si>
+    <t># 修正前                                    # 修正後</t>
+  </si>
+  <si>
+    <t>"slv_com_top_inst.CLK2"                  → "slv_com_top_inst.CLKCOM_OUT"</t>
+  </si>
+  <si>
+    <t>"slv_com_top_inst.CLK2A"                 → "slv_com_top_inst/CLK2A"</t>
+  </si>
+  <si>
+    <t>LPF Section 2, 4, 5, 6 の全8箇所を修正する必要があります。</t>
+  </si>
+  <si>
+    <t>CLK1↔CLKCOM_OUT の59+23パスにMULTICYCLE制約が適用</t>
+  </si>
+  <si>
+    <t>CLKCOM_OUTのタイミング違反が解消される可能性が高い（ルーティング資源の解放）</t>
+  </si>
+  <si>
+    <t>まとめ</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>RTLソース</t>
+  </si>
+  <si>
+    <t>タイミング制約新規作成 (LPF)</t>
+  </si>
+  <si>
+    <t>✓ 適用済み</t>
+  </si>
+  <si>
+    <t>S3IO CLK制約追加 (LPF)</t>
+  </si>
+  <si>
+    <t>RTLデッドコード削除</t>
+  </si>
+  <si>
+    <t>✓ 反映済み</t>
+  </si>
+  <si>
+    <t>(No1-3分析)</t>
+  </si>
+  <si>
+    <t>ワーニング削除 (RTL+FDC)</t>
+  </si>
+  <si>
+    <t>FDC未読込のため一部未反映</t>
+  </si>
+  <si>
+    <t>S3IO通信異常調査</t>
+  </si>
+  <si>
+    <t>✓ 反映済み（LPF部分）</t>
+  </si>
+  <si>
+    <t>No6追加解析</t>
+  </si>
+  <si>
+    <t>ワーニング増加原因解消</t>
+  </si>
+  <si>
+    <t>9-修正1</t>
+  </si>
+  <si>
+    <t>CD134エラー修正</t>
+  </si>
+  <si>
+    <t>✓ 完全反映</t>
+  </si>
+  <si>
+    <t>9-修正2</t>
+  </si>
+  <si>
+    <t>MT420/MT529修正</t>
+  </si>
+  <si>
+    <t>9-修正3</t>
+  </si>
+  <si>
+    <t>CLKCOM_OUTタイミング修正</t>
+  </si>
+  <si>
+    <t>この2点を修正して再コンパイルすれば、FDC制約とLPFタイミング制約が全て有効化され、CLKCOM_OUTのタイミング違反解消が期待できます。修正しますか？</t>
+  </si>
+  <si>
+    <t>Updated todo list tracking modification history and synthesis report review tasks</t>
+  </si>
+  <si>
+    <t>Update Todos</t>
+  </si>
+  <si>
+    <t> Read modification history (修正履歴.xlsx) - items No.1-9</t>
+  </si>
+  <si>
+    <t> Read synthesis report (SP0557_SP0557.srr) for errors/warnings</t>
+  </si>
+  <si>
+    <t> Read place &amp; route / timing reports for MAP/PAR results</t>
+  </si>
+  <si>
+    <t> Verify RTL source files contain the expected changes from No.9 sheet</t>
+  </si>
+  <si>
+    <t> Verify pll_gen.fdc is being loaded by synthesis and check why MT420/MT529 remain</t>
+  </si>
+  <si>
+    <t> Compare previous vs current warning counts</t>
+  </si>
+  <si>
+    <t> Report verification results</t>
+  </si>
+  <si>
+    <t>これはdiamondツール上で実施する手順ではないのですか</t>
+  </si>
+  <si>
+    <t>はい、その通りです。</t>
+  </si>
+  <si>
+    <t>Diamond上での操作手順</t>
+  </si>
+  <si>
+    <t>3. 以下の2ファイルを追加:</t>
+  </si>
+  <si>
+    <t>5. 保存してから再合成（Synthesize）を実行</t>
+  </si>
+  <si>
+    <t>残りの問題: LPFクロックネット名の修正</t>
+  </si>
+  <si>
+    <t>修正前</t>
+  </si>
+  <si>
+    <t>修正後</t>
+  </si>
+  <si>
+    <t>"slv_com_top_inst.CLK2"</t>
+  </si>
+  <si>
+    <t>"slv_com_top_inst.CLKCOM_OUT"</t>
+  </si>
+  <si>
+    <t>"slv_com_top_inst.CLK2A"</t>
+  </si>
+  <si>
+    <t>"slv_com_top_inst/CLK2A"</t>
+  </si>
+  <si>
+    <t>&lt;Source name="RTL/IPcore/pll_gen/pll_gen.fdc" type="FDC" type_short="FDC"&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;Options/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;/Source&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Source name="SP0557/SP0557.fdc" type="FDC" type_short="FDC"&gt;</t>
+  </si>
+  <si>
+    <t>pll_gen.fdc の内容は正しく修正されています:</t>
+  </si>
+  <si>
+    <t>{p:CLKOP} → {n:CLKOP_t} ✓</t>
+  </si>
+  <si>
+    <t>{p:CLKOS} → {n:CLKOS_t} ✓</t>
+  </si>
+  <si>
+    <t>{p:CLKOS2} → {n:CLKOS2_t} ✓</t>
+  </si>
+  <si>
+    <t>{p:CLKOS3} → {n:CLKOS3_t} ✓</t>
+  </si>
+  <si>
+    <t>全クロックが -clockgroup pll_clks で統一 ✓</t>
+  </si>
+  <si>
+    <t>stdout.log にFDCファイル削除の記録:</t>
+  </si>
+  <si>
+    <t>slv_com_top_inst/CLK2A (.ではなく/)</t>
+  </si>
+  <si>
+    <t>CLK1→CLKCOM_OUT: 59パスがFREQUENCY NET "slv_com_top_inst.CLKCOM_OUT" 100MHzで解析（MULTICYCLEなし）</t>
+  </si>
+  <si>
+    <t>CLKCOM_OUT→CLK1: 23パスがFREQUENCY NET "slv_com_top_inst.CLK1" 10MHzで解析（MULTICYCLEなし）</t>
+  </si>
+  <si>
+    <t>Hold違反: CLK1ドメインで -0.321ns（s_LRSTb_r44, TX_RSTb_i_r8）</t>
+  </si>
+  <si>
+    <t>SP0557.ldf に以下の2行を追加する必要があります:</t>
+  </si>
+  <si>
+    <t>こちらは .lpf ファイルのテキスト修正なので、Diamond上でもテキストエディタでもどちらでも対応可能です。修正箇所は以下の通りです:</t>
+  </si>
+  <si>
+    <r>
+      <t>0件</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (合成成功)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1件</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (CLKCOM_OUT: 98.483MHz &lt; 100MHz)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1件</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (CLK1: -0.321ns)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CD134エラー </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>0件</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>根本原因</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: SP0557.ldf（Diamondプロジェクトファイル）に pll_gen.fdc と SP0557.fdc が</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ソースとして登録されていない</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>。VHDLファイルとLPFファイルのみが登録されています。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>結果</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: MT420/MT529ワーニングが</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>5件とも残存</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>適用済み</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (LPF 66行目)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>適用済み</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (LPF 362行目)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>これにより以下の制約が</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>全て無視</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>されています:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>これが</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>CLKCOM_OUTタイミング違反の直接原因</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>です（98.483MHz &lt; 100MHz）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>一部のみ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (ネット名不一致で制約無視)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>一部のみ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (同上)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>✗ 未反映</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (LDFにFDC未登録)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>✗ 未反映</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (ネット名不一致)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>結論</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: RTLソースコードの修正は全て正しく適用されていますが、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>2つの設定上の問題</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>により、コンパイル結果には完全に反映されていません。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1. FDCファイルがDiamondプロジェクトに未登録</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> → MT420/MT529残存</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. LPFのクロックネット名不一致</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (CLK2 ≠ CLKCOM_OUT, .CLK2A ≠ /CLK2A) → MULTICYCLE/BLOCK PATH制約が無視されタイミング違反継続</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SP0557.ldf はDiamond GUIで管理されるプロジェクトファイルなので、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>FDCファイルの登録はDiamond上で行うのが正しい手順</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>です。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1. Diamond</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>でプロジェクト SP0557.ldf を開く</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. File List</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> パネルで右クリック → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>Add</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>Existing File...</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. ファイルタイプが </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>FDC (Synplify Forward Declaration Constraint)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> として認識されていることを確認</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>.ldf をテキストエディタで直接編集しても動作はしますが、Diamondが管理するXML構造なので、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>Diamond GUI上で追加する方が安全</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>です。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>LPF内の </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>Section 2, 4, 5, 6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> の計8箇所が対象です。こちらの修正は私の方で実施できますが、対応しますか？</t>
+    </r>
+  </si>
+  <si>
+    <t>11</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>No1~10の確認</t>
+    <rPh sb="7" eb="9">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="30">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5786,16 +7431,32 @@
       <charset val="128"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
       <name val="Meiryo UI"/>
       <family val="3"/>
       <charset val="128"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Meiryo UI"/>
       <family val="3"/>
       <charset val="128"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -5862,7 +7523,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6112,20 +7773,47 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6586,21 +8274,39 @@
       <c r="F12" s="26"/>
     </row>
     <row r="13" spans="3:6">
-      <c r="C13" s="26"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="27"/>
+      <c r="C13" s="26">
+        <v>9</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>752</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>753</v>
+      </c>
       <c r="F13" s="26"/>
     </row>
     <row r="14" spans="3:6">
-      <c r="C14" s="26"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="27"/>
+      <c r="C14" s="26">
+        <v>10</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>836</v>
+      </c>
+      <c r="E14" s="27" t="s">
+        <v>837</v>
+      </c>
       <c r="F14" s="26"/>
     </row>
     <row r="15" spans="3:6">
-      <c r="C15" s="26"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="27"/>
+      <c r="C15" s="26">
+        <v>11</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E15" s="27" t="s">
+        <v>1020</v>
+      </c>
       <c r="F15" s="26"/>
     </row>
     <row r="16" spans="3:6">
@@ -6706,6 +8412,2165 @@
       <c r="F32" s="26"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14089E9A-DD6C-474E-BC76-1DCDCF7A2A9D}">
+  <dimension ref="A1:B181"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="24">
+      <c r="A1" s="14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="1" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="24">
+      <c r="A7" s="14" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="18.75">
+      <c r="A9" s="15" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="1" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="18.75">
+      <c r="A13" s="15" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="17" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="18"/>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="18" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="24" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="18" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="1" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="16" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="16" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="1" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" s="16" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" s="16" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" s="17" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="18"/>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="18" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" s="18" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="1" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" s="16" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" s="1" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" s="16" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="17" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" s="18"/>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" s="18" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" s="24" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" s="18" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="1" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="16" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="16" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" s="16" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" s="16" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" s="1" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" s="16" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="16" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" s="16" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" s="16" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" s="16" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" s="16" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="16" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" s="16" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" s="16" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" s="16" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" s="16" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" s="16" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" s="16" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" s="16" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" s="16" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" s="16" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" s="16" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" s="16" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="16" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" s="16" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" s="16" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" s="16" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" s="16" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" s="16" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" s="16" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" s="16" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" s="16" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" s="16" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" s="16" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" s="16" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128" s="16" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" s="16" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" s="16" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133" s="16" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1">
+      <c r="A136" s="16" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1">
+      <c r="A137" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138" s="16" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1">
+      <c r="A139" s="16" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1">
+      <c r="A141" s="17" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" ht="24">
+      <c r="A145" s="14" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" ht="18.75">
+      <c r="A147" s="15" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" s="1" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" s="18"/>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" s="18" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" s="18" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" s="18" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" s="1" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" ht="24">
+      <c r="A159" s="14" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B161" s="20" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" ht="71.25">
+      <c r="A162" s="21" t="s">
+        <v>772</v>
+      </c>
+      <c r="B162" s="9" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" ht="71.25">
+      <c r="A163" s="21" t="s">
+        <v>774</v>
+      </c>
+      <c r="B163" s="9" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" ht="71.25">
+      <c r="A164" s="21" t="s">
+        <v>776</v>
+      </c>
+      <c r="B164" s="9" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" ht="60">
+      <c r="A165" s="21" t="s">
+        <v>778</v>
+      </c>
+      <c r="B165" s="21" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" ht="47.25">
+      <c r="A166" s="21" t="s">
+        <v>779</v>
+      </c>
+      <c r="B166" s="9" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" ht="24">
+      <c r="A169" s="14" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="1" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="18"/>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="19" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="19" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="88" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="19" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1">
+      <c r="A177" s="19" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1">
+      <c r="A178" s="19" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1">
+      <c r="A179" s="19" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1">
+      <c r="A180" s="25" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1">
+      <c r="A181" s="25" t="s">
+        <v>783</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80AF1D6C-FC01-45A2-8677-95498AA084BB}">
+  <dimension ref="A1:E149"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="1" max="1" width="77.75" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="5" max="5" width="7.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A1" s="89" t="s">
+        <v>839</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+    </row>
+    <row r="2" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A2" s="74" t="s">
+        <v>840</v>
+      </c>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+    </row>
+    <row r="3" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A3" s="72"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+    </row>
+    <row r="4" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A4" s="89" t="s">
+        <v>841</v>
+      </c>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+    </row>
+    <row r="5" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A5" s="91" t="s">
+        <v>842</v>
+      </c>
+      <c r="B5" s="92" t="s">
+        <v>557</v>
+      </c>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+    </row>
+    <row r="6" spans="1:5" s="90" customFormat="1" ht="20.25" thickBot="1">
+      <c r="A6" s="79" t="s">
+        <v>843</v>
+      </c>
+      <c r="B6" s="93" t="s">
+        <v>996</v>
+      </c>
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
+    </row>
+    <row r="7" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A7" s="79" t="s">
+        <v>844</v>
+      </c>
+      <c r="B7" s="93" t="s">
+        <v>997</v>
+      </c>
+      <c r="C7" s="72"/>
+      <c r="D7" s="72"/>
+      <c r="E7" s="72"/>
+    </row>
+    <row r="8" spans="1:5" s="90" customFormat="1" ht="20.25" thickBot="1">
+      <c r="A8" s="79" t="s">
+        <v>845</v>
+      </c>
+      <c r="B8" s="93" t="s">
+        <v>998</v>
+      </c>
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+    </row>
+    <row r="9" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A9" s="79" t="s">
+        <v>846</v>
+      </c>
+      <c r="B9" s="89" t="s">
+        <v>847</v>
+      </c>
+      <c r="C9" s="72"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="72"/>
+    </row>
+    <row r="10" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A10" s="72"/>
+      <c r="B10" s="72"/>
+      <c r="C10" s="72"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="72"/>
+    </row>
+    <row r="11" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A11" s="89" t="s">
+        <v>848</v>
+      </c>
+      <c r="B11" s="72"/>
+      <c r="C11" s="72"/>
+      <c r="D11" s="72"/>
+      <c r="E11" s="72"/>
+    </row>
+    <row r="12" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A12" s="89" t="s">
+        <v>849</v>
+      </c>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+    </row>
+    <row r="13" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A13" s="91" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="91" t="s">
+        <v>658</v>
+      </c>
+      <c r="C13" s="91" t="s">
+        <v>850</v>
+      </c>
+      <c r="D13" s="92" t="s">
+        <v>851</v>
+      </c>
+      <c r="E13" s="72"/>
+    </row>
+    <row r="14" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A14" s="79" t="s">
+        <v>852</v>
+      </c>
+      <c r="B14" s="79" t="s">
+        <v>853</v>
+      </c>
+      <c r="C14" s="94" t="s">
+        <v>854</v>
+      </c>
+      <c r="D14" s="81" t="s">
+        <v>999</v>
+      </c>
+      <c r="E14" s="72"/>
+    </row>
+    <row r="15" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A15" s="79" t="s">
+        <v>855</v>
+      </c>
+      <c r="B15" s="79" t="s">
+        <v>856</v>
+      </c>
+      <c r="C15" s="94" t="s">
+        <v>854</v>
+      </c>
+      <c r="D15" s="81" t="s">
+        <v>999</v>
+      </c>
+      <c r="E15" s="72"/>
+    </row>
+    <row r="16" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A16" s="79" t="s">
+        <v>857</v>
+      </c>
+      <c r="B16" s="79" t="s">
+        <v>858</v>
+      </c>
+      <c r="C16" s="94" t="s">
+        <v>854</v>
+      </c>
+      <c r="D16" s="74" t="s">
+        <v>999</v>
+      </c>
+      <c r="E16" s="72"/>
+    </row>
+    <row r="17" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A17" s="74" t="s">
+        <v>859</v>
+      </c>
+      <c r="B17" s="72"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="72"/>
+      <c r="E17" s="72"/>
+    </row>
+    <row r="18" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A18" s="72"/>
+      <c r="B18" s="72"/>
+      <c r="C18" s="72"/>
+      <c r="D18" s="72"/>
+      <c r="E18" s="72"/>
+    </row>
+    <row r="19" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A19" s="89" t="s">
+        <v>860</v>
+      </c>
+      <c r="B19" s="72"/>
+      <c r="C19" s="72"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+    </row>
+    <row r="20" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A20" s="74" t="s">
+        <v>983</v>
+      </c>
+      <c r="B20" s="72"/>
+      <c r="C20" s="72"/>
+      <c r="D20" s="72"/>
+      <c r="E20" s="72"/>
+    </row>
+    <row r="21" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A21" s="75"/>
+      <c r="B21" s="72"/>
+      <c r="C21" s="72"/>
+      <c r="D21" s="72"/>
+      <c r="E21" s="72"/>
+    </row>
+    <row r="22" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A22" s="75" t="s">
+        <v>984</v>
+      </c>
+      <c r="B22" s="72"/>
+      <c r="C22" s="72"/>
+      <c r="D22" s="72"/>
+      <c r="E22" s="72"/>
+    </row>
+    <row r="23" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A23" s="75" t="s">
+        <v>985</v>
+      </c>
+      <c r="B23" s="72"/>
+      <c r="C23" s="72"/>
+      <c r="D23" s="72"/>
+      <c r="E23" s="72"/>
+    </row>
+    <row r="24" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A24" s="75" t="s">
+        <v>986</v>
+      </c>
+      <c r="B24" s="72"/>
+      <c r="C24" s="72"/>
+      <c r="D24" s="72"/>
+      <c r="E24" s="72"/>
+    </row>
+    <row r="25" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A25" s="75" t="s">
+        <v>987</v>
+      </c>
+      <c r="B25" s="72"/>
+      <c r="C25" s="72"/>
+      <c r="D25" s="72"/>
+      <c r="E25" s="72"/>
+    </row>
+    <row r="26" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A26" s="75" t="s">
+        <v>988</v>
+      </c>
+      <c r="B26" s="72"/>
+      <c r="C26" s="72"/>
+      <c r="D26" s="72"/>
+      <c r="E26" s="72"/>
+    </row>
+    <row r="27" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A27" s="74"/>
+      <c r="B27" s="72"/>
+      <c r="C27" s="72"/>
+      <c r="D27" s="72"/>
+      <c r="E27" s="72"/>
+    </row>
+    <row r="28" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A28" s="89" t="s">
+        <v>861</v>
+      </c>
+      <c r="B28" s="72"/>
+      <c r="C28" s="72"/>
+      <c r="D28" s="72"/>
+      <c r="E28" s="72"/>
+    </row>
+    <row r="29" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A29" s="74" t="s">
+        <v>862</v>
+      </c>
+      <c r="B29" s="72"/>
+      <c r="C29" s="72"/>
+      <c r="D29" s="72"/>
+      <c r="E29" s="72"/>
+    </row>
+    <row r="30" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A30" s="72" t="s">
+        <v>863</v>
+      </c>
+      <c r="B30" s="72"/>
+      <c r="C30" s="72"/>
+      <c r="D30" s="72"/>
+      <c r="E30" s="72"/>
+    </row>
+    <row r="31" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A31" s="74" t="s">
+        <v>989</v>
+      </c>
+      <c r="B31" s="72"/>
+      <c r="C31" s="72"/>
+      <c r="D31" s="72"/>
+      <c r="E31" s="72"/>
+    </row>
+    <row r="32" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A32" s="72" t="s">
+        <v>864</v>
+      </c>
+      <c r="B32" s="72"/>
+      <c r="C32" s="72"/>
+      <c r="D32" s="72"/>
+      <c r="E32" s="72"/>
+    </row>
+    <row r="33" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A33" s="72" t="s">
+        <v>865</v>
+      </c>
+      <c r="B33" s="72"/>
+      <c r="C33" s="72"/>
+      <c r="D33" s="72"/>
+      <c r="E33" s="72"/>
+    </row>
+    <row r="34" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A34" s="89" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B34" s="72"/>
+      <c r="C34" s="72"/>
+      <c r="D34" s="72"/>
+      <c r="E34" s="72"/>
+    </row>
+    <row r="35" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A35" s="89" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B35" s="72"/>
+      <c r="C35" s="72"/>
+      <c r="D35" s="72"/>
+      <c r="E35" s="72"/>
+    </row>
+    <row r="36" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A36" s="72" t="s">
+        <v>866</v>
+      </c>
+      <c r="B36" s="72"/>
+      <c r="C36" s="72"/>
+      <c r="D36" s="72"/>
+      <c r="E36" s="72"/>
+    </row>
+    <row r="37" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A37" s="72" t="s">
+        <v>867</v>
+      </c>
+      <c r="B37" s="72"/>
+      <c r="C37" s="72"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="72"/>
+    </row>
+    <row r="38" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A38" s="72" t="s">
+        <v>868</v>
+      </c>
+      <c r="B38" s="72"/>
+      <c r="C38" s="72"/>
+      <c r="D38" s="72"/>
+      <c r="E38" s="72"/>
+    </row>
+    <row r="39" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A39" s="72" t="s">
+        <v>869</v>
+      </c>
+      <c r="B39" s="72"/>
+      <c r="C39" s="72"/>
+      <c r="D39" s="72"/>
+      <c r="E39" s="72"/>
+    </row>
+    <row r="40" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A40" s="72" t="s">
+        <v>870</v>
+      </c>
+      <c r="B40" s="72"/>
+      <c r="C40" s="72"/>
+      <c r="D40" s="72"/>
+      <c r="E40" s="72"/>
+    </row>
+    <row r="41" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A41" s="74" t="s">
+        <v>871</v>
+      </c>
+      <c r="B41" s="72"/>
+      <c r="C41" s="72"/>
+      <c r="D41" s="72"/>
+      <c r="E41" s="72"/>
+    </row>
+    <row r="42" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A42" s="72"/>
+      <c r="B42" s="72"/>
+      <c r="C42" s="72"/>
+      <c r="D42" s="72"/>
+      <c r="E42" s="72"/>
+    </row>
+    <row r="43" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A43" s="89" t="s">
+        <v>872</v>
+      </c>
+      <c r="B43" s="72"/>
+      <c r="C43" s="72"/>
+      <c r="D43" s="72"/>
+      <c r="E43" s="72"/>
+    </row>
+    <row r="44" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A44" s="91" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44" s="92" t="s">
+        <v>71</v>
+      </c>
+      <c r="C44" s="72"/>
+      <c r="D44" s="72"/>
+      <c r="E44" s="72"/>
+    </row>
+    <row r="45" spans="1:5" s="90" customFormat="1" ht="20.25" thickBot="1">
+      <c r="A45" s="79" t="s">
+        <v>873</v>
+      </c>
+      <c r="B45" s="93" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C45" s="72"/>
+      <c r="D45" s="72"/>
+      <c r="E45" s="72"/>
+    </row>
+    <row r="46" spans="1:5" s="90" customFormat="1" ht="20.25" thickBot="1">
+      <c r="A46" s="79" t="s">
+        <v>874</v>
+      </c>
+      <c r="B46" s="93" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C46" s="72"/>
+      <c r="D46" s="72"/>
+      <c r="E46" s="72"/>
+    </row>
+    <row r="47" spans="1:5" s="90" customFormat="1" ht="20.25" thickBot="1">
+      <c r="A47" s="79" t="s">
+        <v>875</v>
+      </c>
+      <c r="B47" s="93" t="s">
+        <v>876</v>
+      </c>
+      <c r="C47" s="72"/>
+      <c r="D47" s="72"/>
+      <c r="E47" s="72"/>
+    </row>
+    <row r="48" spans="1:5" s="90" customFormat="1" ht="20.25" thickBot="1">
+      <c r="A48" s="79" t="s">
+        <v>877</v>
+      </c>
+      <c r="B48" s="93" t="s">
+        <v>876</v>
+      </c>
+      <c r="C48" s="72"/>
+      <c r="D48" s="72"/>
+      <c r="E48" s="72"/>
+    </row>
+    <row r="49" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A49" s="79" t="s">
+        <v>878</v>
+      </c>
+      <c r="B49" s="89" t="s">
+        <v>876</v>
+      </c>
+      <c r="C49" s="72"/>
+      <c r="D49" s="72"/>
+      <c r="E49" s="72"/>
+    </row>
+    <row r="50" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A50" s="89" t="s">
+        <v>879</v>
+      </c>
+      <c r="B50" s="72"/>
+      <c r="C50" s="72"/>
+      <c r="D50" s="72"/>
+      <c r="E50" s="72"/>
+    </row>
+    <row r="51" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A51" s="91" t="s">
+        <v>880</v>
+      </c>
+      <c r="B51" s="91" t="s">
+        <v>881</v>
+      </c>
+      <c r="C51" s="92" t="s">
+        <v>71</v>
+      </c>
+      <c r="D51" s="72"/>
+      <c r="E51" s="72"/>
+    </row>
+    <row r="52" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A52" s="79" t="s">
+        <v>882</v>
+      </c>
+      <c r="B52" s="79" t="s">
+        <v>883</v>
+      </c>
+      <c r="C52" s="93" t="s">
+        <v>884</v>
+      </c>
+      <c r="D52" s="72"/>
+      <c r="E52" s="72"/>
+    </row>
+    <row r="53" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A53" s="79" t="s">
+        <v>885</v>
+      </c>
+      <c r="B53" s="79" t="s">
+        <v>990</v>
+      </c>
+      <c r="C53" s="89" t="s">
+        <v>884</v>
+      </c>
+      <c r="D53" s="72"/>
+      <c r="E53" s="72"/>
+    </row>
+    <row r="54" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A54" s="74" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B54" s="72"/>
+      <c r="C54" s="72"/>
+      <c r="D54" s="72"/>
+      <c r="E54" s="72"/>
+    </row>
+    <row r="55" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A55" s="91" t="s">
+        <v>886</v>
+      </c>
+      <c r="B55" s="91" t="s">
+        <v>887</v>
+      </c>
+      <c r="C55" s="92" t="s">
+        <v>888</v>
+      </c>
+      <c r="D55" s="72"/>
+      <c r="E55" s="72"/>
+    </row>
+    <row r="56" spans="1:5" s="90" customFormat="1" ht="132.75" thickBot="1">
+      <c r="A56" s="79" t="s">
+        <v>889</v>
+      </c>
+      <c r="B56" s="79" t="s">
+        <v>890</v>
+      </c>
+      <c r="C56" s="81" t="s">
+        <v>891</v>
+      </c>
+      <c r="D56" s="72"/>
+      <c r="E56" s="72"/>
+    </row>
+    <row r="57" spans="1:5" s="90" customFormat="1" ht="83.25" thickBot="1">
+      <c r="A57" s="79" t="s">
+        <v>892</v>
+      </c>
+      <c r="B57" s="79" t="s">
+        <v>893</v>
+      </c>
+      <c r="C57" s="81" t="s">
+        <v>894</v>
+      </c>
+      <c r="D57" s="72"/>
+      <c r="E57" s="72"/>
+    </row>
+    <row r="58" spans="1:5" s="90" customFormat="1" ht="99.75" thickBot="1">
+      <c r="A58" s="94" t="s">
+        <v>895</v>
+      </c>
+      <c r="B58" s="94" t="s">
+        <v>896</v>
+      </c>
+      <c r="C58" s="93" t="s">
+        <v>897</v>
+      </c>
+      <c r="D58" s="72"/>
+      <c r="E58" s="72"/>
+    </row>
+    <row r="59" spans="1:5" s="90" customFormat="1" ht="66">
+      <c r="A59" s="79" t="s">
+        <v>898</v>
+      </c>
+      <c r="B59" s="79" t="s">
+        <v>899</v>
+      </c>
+      <c r="C59" s="74" t="s">
+        <v>900</v>
+      </c>
+      <c r="D59" s="72"/>
+      <c r="E59" s="72"/>
+    </row>
+    <row r="60" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A60" s="89" t="s">
+        <v>901</v>
+      </c>
+      <c r="B60" s="72"/>
+      <c r="C60" s="72"/>
+      <c r="D60" s="72"/>
+      <c r="E60" s="72"/>
+    </row>
+    <row r="61" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A61" s="74" t="s">
+        <v>991</v>
+      </c>
+      <c r="B61" s="72"/>
+      <c r="C61" s="72"/>
+      <c r="D61" s="72"/>
+      <c r="E61" s="72"/>
+    </row>
+    <row r="62" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A62" s="74" t="s">
+        <v>992</v>
+      </c>
+      <c r="B62" s="72"/>
+      <c r="C62" s="72"/>
+      <c r="D62" s="72"/>
+      <c r="E62" s="72"/>
+    </row>
+    <row r="63" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A63" s="74" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B63" s="72"/>
+      <c r="C63" s="72"/>
+      <c r="D63" s="72"/>
+      <c r="E63" s="72"/>
+    </row>
+    <row r="64" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A64" s="72"/>
+      <c r="B64" s="72"/>
+      <c r="C64" s="72"/>
+      <c r="D64" s="72"/>
+      <c r="E64" s="72"/>
+    </row>
+    <row r="65" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A65" s="89" t="s">
+        <v>902</v>
+      </c>
+      <c r="B65" s="72"/>
+      <c r="C65" s="72"/>
+      <c r="D65" s="72"/>
+      <c r="E65" s="72"/>
+    </row>
+    <row r="66" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A66" s="91" t="s">
+        <v>903</v>
+      </c>
+      <c r="B66" s="91" t="s">
+        <v>887</v>
+      </c>
+      <c r="C66" s="91" t="s">
+        <v>904</v>
+      </c>
+      <c r="D66" s="91" t="s">
+        <v>905</v>
+      </c>
+      <c r="E66" s="92" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A67" s="79" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67" s="79" t="s">
+        <v>906</v>
+      </c>
+      <c r="C67" s="79" t="s">
+        <v>907</v>
+      </c>
+      <c r="D67" s="94" t="s">
+        <v>908</v>
+      </c>
+      <c r="E67" s="93" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A68" s="79" t="s">
+        <v>910</v>
+      </c>
+      <c r="B68" s="79" t="s">
+        <v>906</v>
+      </c>
+      <c r="C68" s="79" t="s">
+        <v>911</v>
+      </c>
+      <c r="D68" s="79" t="s">
+        <v>912</v>
+      </c>
+      <c r="E68" s="81" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A69" s="79" t="s">
+        <v>101</v>
+      </c>
+      <c r="B69" s="79" t="s">
+        <v>914</v>
+      </c>
+      <c r="C69" s="79" t="s">
+        <v>915</v>
+      </c>
+      <c r="D69" s="79" t="s">
+        <v>916</v>
+      </c>
+      <c r="E69" s="81" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A70" s="79" t="s">
+        <v>917</v>
+      </c>
+      <c r="B70" s="79" t="s">
+        <v>918</v>
+      </c>
+      <c r="C70" s="79" t="s">
+        <v>919</v>
+      </c>
+      <c r="D70" s="79" t="s">
+        <v>916</v>
+      </c>
+      <c r="E70" s="81" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A71" s="79" t="s">
+        <v>920</v>
+      </c>
+      <c r="B71" s="79" t="s">
+        <v>510</v>
+      </c>
+      <c r="C71" s="79" t="s">
+        <v>510</v>
+      </c>
+      <c r="D71" s="79" t="s">
+        <v>510</v>
+      </c>
+      <c r="E71" s="74" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A72" s="74" t="s">
+        <v>993</v>
+      </c>
+      <c r="B72" s="72"/>
+      <c r="C72" s="72"/>
+      <c r="D72" s="72"/>
+      <c r="E72" s="72"/>
+    </row>
+    <row r="73" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A73" s="72"/>
+      <c r="B73" s="72"/>
+      <c r="C73" s="72"/>
+      <c r="D73" s="72"/>
+      <c r="E73" s="72"/>
+    </row>
+    <row r="74" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A74" s="89" t="s">
+        <v>922</v>
+      </c>
+      <c r="B74" s="72"/>
+      <c r="C74" s="72"/>
+      <c r="D74" s="72"/>
+      <c r="E74" s="72"/>
+    </row>
+    <row r="75" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A75" s="89" t="s">
+        <v>923</v>
+      </c>
+      <c r="B75" s="72"/>
+      <c r="C75" s="72"/>
+      <c r="D75" s="72"/>
+      <c r="E75" s="72"/>
+    </row>
+    <row r="76" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A76" s="74" t="s">
+        <v>994</v>
+      </c>
+      <c r="B76" s="72"/>
+      <c r="C76" s="72"/>
+      <c r="D76" s="72"/>
+      <c r="E76" s="72"/>
+    </row>
+    <row r="77" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A77" s="72" t="s">
+        <v>979</v>
+      </c>
+      <c r="B77" s="72"/>
+      <c r="C77" s="72"/>
+      <c r="D77" s="72"/>
+      <c r="E77" s="72"/>
+    </row>
+    <row r="78" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A78" s="72" t="s">
+        <v>980</v>
+      </c>
+      <c r="B78" s="72"/>
+      <c r="C78" s="72"/>
+      <c r="D78" s="72"/>
+      <c r="E78" s="72"/>
+    </row>
+    <row r="79" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A79" s="72" t="s">
+        <v>981</v>
+      </c>
+      <c r="B79" s="72"/>
+      <c r="C79" s="72"/>
+      <c r="D79" s="72"/>
+      <c r="E79" s="72"/>
+    </row>
+    <row r="80" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A80" s="72" t="s">
+        <v>982</v>
+      </c>
+      <c r="B80" s="72"/>
+      <c r="C80" s="72"/>
+      <c r="D80" s="72"/>
+      <c r="E80" s="72"/>
+    </row>
+    <row r="81" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A81" s="72" t="s">
+        <v>980</v>
+      </c>
+      <c r="B81" s="72"/>
+      <c r="C81" s="72"/>
+      <c r="D81" s="72"/>
+      <c r="E81" s="72"/>
+    </row>
+    <row r="82" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A82" s="72" t="s">
+        <v>981</v>
+      </c>
+      <c r="B82" s="72"/>
+      <c r="C82" s="72"/>
+      <c r="D82" s="72"/>
+      <c r="E82" s="72"/>
+    </row>
+    <row r="83" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A83" s="74" t="s">
+        <v>924</v>
+      </c>
+      <c r="B83" s="72"/>
+      <c r="C83" s="72"/>
+      <c r="D83" s="72"/>
+      <c r="E83" s="72"/>
+    </row>
+    <row r="84" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A84" s="75"/>
+      <c r="B84" s="72"/>
+      <c r="C84" s="72"/>
+      <c r="D84" s="72"/>
+      <c r="E84" s="72"/>
+    </row>
+    <row r="85" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A85" s="75" t="s">
+        <v>925</v>
+      </c>
+      <c r="B85" s="72"/>
+      <c r="C85" s="72"/>
+      <c r="D85" s="72"/>
+      <c r="E85" s="72"/>
+    </row>
+    <row r="86" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A86" s="75" t="s">
+        <v>926</v>
+      </c>
+      <c r="B86" s="72"/>
+      <c r="C86" s="72"/>
+      <c r="D86" s="72"/>
+      <c r="E86" s="72"/>
+    </row>
+    <row r="87" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A87" s="75" t="s">
+        <v>927</v>
+      </c>
+      <c r="B87" s="72"/>
+      <c r="C87" s="72"/>
+      <c r="D87" s="72"/>
+      <c r="E87" s="72"/>
+    </row>
+    <row r="88" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A88" s="74"/>
+      <c r="B88" s="72"/>
+      <c r="C88" s="72"/>
+      <c r="D88" s="72"/>
+      <c r="E88" s="72"/>
+    </row>
+    <row r="89" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A89" s="89" t="s">
+        <v>928</v>
+      </c>
+      <c r="B89" s="72"/>
+      <c r="C89" s="72"/>
+      <c r="D89" s="72"/>
+      <c r="E89" s="72"/>
+    </row>
+    <row r="90" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A90" s="72" t="s">
+        <v>929</v>
+      </c>
+      <c r="B90" s="72"/>
+      <c r="C90" s="72"/>
+      <c r="D90" s="72"/>
+      <c r="E90" s="72"/>
+    </row>
+    <row r="91" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A91" s="72" t="s">
+        <v>930</v>
+      </c>
+      <c r="B91" s="72"/>
+      <c r="C91" s="72"/>
+      <c r="D91" s="72"/>
+      <c r="E91" s="72"/>
+    </row>
+    <row r="92" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A92" s="72" t="s">
+        <v>931</v>
+      </c>
+      <c r="B92" s="72"/>
+      <c r="C92" s="72"/>
+      <c r="D92" s="72"/>
+      <c r="E92" s="72"/>
+    </row>
+    <row r="93" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A93" s="74" t="s">
+        <v>932</v>
+      </c>
+      <c r="B93" s="72"/>
+      <c r="C93" s="72"/>
+      <c r="D93" s="72"/>
+      <c r="E93" s="72"/>
+    </row>
+    <row r="94" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A94" s="74" t="s">
+        <v>924</v>
+      </c>
+      <c r="B94" s="72"/>
+      <c r="C94" s="72"/>
+      <c r="D94" s="72"/>
+      <c r="E94" s="72"/>
+    </row>
+    <row r="95" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A95" s="75"/>
+      <c r="B95" s="72"/>
+      <c r="C95" s="72"/>
+      <c r="D95" s="72"/>
+      <c r="E95" s="72"/>
+    </row>
+    <row r="96" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A96" s="75" t="s">
+        <v>933</v>
+      </c>
+      <c r="B96" s="72"/>
+      <c r="C96" s="72"/>
+      <c r="D96" s="72"/>
+      <c r="E96" s="72"/>
+    </row>
+    <row r="97" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A97" s="75" t="s">
+        <v>934</v>
+      </c>
+      <c r="B97" s="72"/>
+      <c r="C97" s="72"/>
+      <c r="D97" s="72"/>
+      <c r="E97" s="72"/>
+    </row>
+    <row r="98" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A98" s="74"/>
+      <c r="B98" s="72"/>
+      <c r="C98" s="72"/>
+      <c r="D98" s="72"/>
+      <c r="E98" s="72"/>
+    </row>
+    <row r="99" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A99" s="72"/>
+      <c r="B99" s="72"/>
+      <c r="C99" s="72"/>
+      <c r="D99" s="72"/>
+      <c r="E99" s="72"/>
+    </row>
+    <row r="100" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A100" s="89" t="s">
+        <v>935</v>
+      </c>
+      <c r="B100" s="72"/>
+      <c r="C100" s="72"/>
+      <c r="D100" s="72"/>
+      <c r="E100" s="72"/>
+    </row>
+    <row r="101" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A101" s="91" t="s">
+        <v>936</v>
+      </c>
+      <c r="B101" s="91" t="s">
+        <v>658</v>
+      </c>
+      <c r="C101" s="91" t="s">
+        <v>937</v>
+      </c>
+      <c r="D101" s="92" t="s">
+        <v>851</v>
+      </c>
+      <c r="E101" s="72"/>
+    </row>
+    <row r="102" spans="1:5" s="90" customFormat="1" ht="83.25" thickBot="1">
+      <c r="A102" s="79">
+        <v>1</v>
+      </c>
+      <c r="B102" s="79" t="s">
+        <v>938</v>
+      </c>
+      <c r="C102" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D102" s="93" t="s">
+        <v>1006</v>
+      </c>
+      <c r="E102" s="72"/>
+    </row>
+    <row r="103" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A103" s="79">
+        <v>2</v>
+      </c>
+      <c r="B103" s="79" t="s">
+        <v>940</v>
+      </c>
+      <c r="C103" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D103" s="93" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E103" s="72"/>
+    </row>
+    <row r="104" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A104" s="79">
+        <v>3</v>
+      </c>
+      <c r="B104" s="79" t="s">
+        <v>941</v>
+      </c>
+      <c r="C104" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D104" s="81" t="s">
+        <v>942</v>
+      </c>
+      <c r="E104" s="72"/>
+    </row>
+    <row r="105" spans="1:5" s="90" customFormat="1" ht="20.25" thickBot="1">
+      <c r="A105" s="79">
+        <v>4</v>
+      </c>
+      <c r="B105" s="79" t="s">
+        <v>943</v>
+      </c>
+      <c r="C105" s="79" t="s">
+        <v>510</v>
+      </c>
+      <c r="D105" s="81" t="s">
+        <v>510</v>
+      </c>
+      <c r="E105" s="72"/>
+    </row>
+    <row r="106" spans="1:5" s="90" customFormat="1" ht="66.75" thickBot="1">
+      <c r="A106" s="79">
+        <v>5</v>
+      </c>
+      <c r="B106" s="79" t="s">
+        <v>944</v>
+      </c>
+      <c r="C106" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D106" s="93" t="s">
+        <v>945</v>
+      </c>
+      <c r="E106" s="72"/>
+    </row>
+    <row r="107" spans="1:5" s="90" customFormat="1" ht="66.75" thickBot="1">
+      <c r="A107" s="79">
+        <v>6</v>
+      </c>
+      <c r="B107" s="79" t="s">
+        <v>946</v>
+      </c>
+      <c r="C107" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D107" s="81" t="s">
+        <v>947</v>
+      </c>
+      <c r="E107" s="72"/>
+    </row>
+    <row r="108" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A108" s="79">
+        <v>7</v>
+      </c>
+      <c r="B108" s="79" t="s">
+        <v>948</v>
+      </c>
+      <c r="C108" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D108" s="81" t="s">
+        <v>942</v>
+      </c>
+      <c r="E108" s="72"/>
+    </row>
+    <row r="109" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A109" s="79">
+        <v>8</v>
+      </c>
+      <c r="B109" s="79" t="s">
+        <v>949</v>
+      </c>
+      <c r="C109" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D109" s="81" t="s">
+        <v>942</v>
+      </c>
+      <c r="E109" s="72"/>
+    </row>
+    <row r="110" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A110" s="79" t="s">
+        <v>950</v>
+      </c>
+      <c r="B110" s="79" t="s">
+        <v>951</v>
+      </c>
+      <c r="C110" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D110" s="93" t="s">
+        <v>952</v>
+      </c>
+      <c r="E110" s="72"/>
+    </row>
+    <row r="111" spans="1:5" s="90" customFormat="1" ht="66.75" thickBot="1">
+      <c r="A111" s="79" t="s">
+        <v>953</v>
+      </c>
+      <c r="B111" s="79" t="s">
+        <v>954</v>
+      </c>
+      <c r="C111" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D111" s="93" t="s">
+        <v>1008</v>
+      </c>
+      <c r="E111" s="72"/>
+    </row>
+    <row r="112" spans="1:5" s="90" customFormat="1" ht="66">
+      <c r="A112" s="79" t="s">
+        <v>955</v>
+      </c>
+      <c r="B112" s="79" t="s">
+        <v>956</v>
+      </c>
+      <c r="C112" s="79" t="s">
+        <v>939</v>
+      </c>
+      <c r="D112" s="89" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E112" s="72"/>
+    </row>
+    <row r="113" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A113" s="89" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B113" s="72"/>
+      <c r="C113" s="72"/>
+      <c r="D113" s="72"/>
+      <c r="E113" s="72"/>
+    </row>
+    <row r="114" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A114" s="75"/>
+      <c r="B114" s="72"/>
+      <c r="C114" s="72"/>
+      <c r="D114" s="72"/>
+      <c r="E114" s="72"/>
+    </row>
+    <row r="115" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A115" s="95" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B115" s="72"/>
+      <c r="C115" s="72"/>
+      <c r="D115" s="72"/>
+      <c r="E115" s="72"/>
+    </row>
+    <row r="116" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A116" s="95" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B116" s="72"/>
+      <c r="C116" s="72"/>
+      <c r="D116" s="72"/>
+      <c r="E116" s="72"/>
+    </row>
+    <row r="117" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A117" s="74"/>
+      <c r="B117" s="72"/>
+      <c r="C117" s="72"/>
+      <c r="D117" s="72"/>
+      <c r="E117" s="72"/>
+    </row>
+    <row r="118" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A118" s="74" t="s">
+        <v>957</v>
+      </c>
+      <c r="B118" s="72"/>
+      <c r="C118" s="72"/>
+      <c r="D118" s="72"/>
+      <c r="E118" s="72"/>
+    </row>
+    <row r="119" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A119" s="74" t="s">
+        <v>958</v>
+      </c>
+      <c r="B119" s="72"/>
+      <c r="C119" s="72"/>
+      <c r="D119" s="72"/>
+      <c r="E119" s="72"/>
+    </row>
+    <row r="120" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A120" s="74" t="s">
+        <v>958</v>
+      </c>
+      <c r="B120" s="72"/>
+      <c r="C120" s="72"/>
+      <c r="D120" s="72"/>
+      <c r="E120" s="72"/>
+    </row>
+    <row r="121" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A121" s="74" t="s">
+        <v>959</v>
+      </c>
+      <c r="B121" s="72"/>
+      <c r="C121" s="72"/>
+      <c r="D121" s="72"/>
+      <c r="E121" s="72"/>
+    </row>
+    <row r="122" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A122" s="74" t="s">
+        <v>960</v>
+      </c>
+      <c r="B122" s="72"/>
+      <c r="C122" s="72"/>
+      <c r="D122" s="72"/>
+      <c r="E122" s="72"/>
+    </row>
+    <row r="123" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A123" s="74" t="s">
+        <v>961</v>
+      </c>
+      <c r="B123" s="72"/>
+      <c r="C123" s="72"/>
+      <c r="D123" s="72"/>
+      <c r="E123" s="72"/>
+    </row>
+    <row r="124" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A124" s="74" t="s">
+        <v>962</v>
+      </c>
+      <c r="B124" s="72"/>
+      <c r="C124" s="72"/>
+      <c r="D124" s="72"/>
+      <c r="E124" s="72"/>
+    </row>
+    <row r="125" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A125" s="74" t="s">
+        <v>963</v>
+      </c>
+      <c r="B125" s="72"/>
+      <c r="C125" s="72"/>
+      <c r="D125" s="72"/>
+      <c r="E125" s="72"/>
+    </row>
+    <row r="126" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A126" s="74" t="s">
+        <v>964</v>
+      </c>
+      <c r="B126" s="72"/>
+      <c r="C126" s="72"/>
+      <c r="D126" s="72"/>
+      <c r="E126" s="72"/>
+    </row>
+    <row r="127" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A127" s="74" t="s">
+        <v>965</v>
+      </c>
+      <c r="B127" s="72"/>
+      <c r="C127" s="72"/>
+      <c r="D127" s="72"/>
+      <c r="E127" s="72"/>
+    </row>
+    <row r="128" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A128" s="74" t="s">
+        <v>966</v>
+      </c>
+      <c r="B128" s="72"/>
+      <c r="C128" s="72"/>
+      <c r="D128" s="72"/>
+      <c r="E128" s="72"/>
+    </row>
+    <row r="129" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A129" s="74" t="s">
+        <v>838</v>
+      </c>
+      <c r="B129" s="72"/>
+      <c r="C129" s="72"/>
+      <c r="D129" s="72"/>
+      <c r="E129" s="72"/>
+    </row>
+    <row r="130" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A130" s="74" t="s">
+        <v>967</v>
+      </c>
+      <c r="B130" s="72"/>
+      <c r="C130" s="72"/>
+      <c r="D130" s="72"/>
+      <c r="E130" s="72"/>
+    </row>
+    <row r="131" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A131" s="74" t="s">
+        <v>968</v>
+      </c>
+      <c r="B131" s="72"/>
+      <c r="C131" s="72"/>
+      <c r="D131" s="72"/>
+      <c r="E131" s="72"/>
+    </row>
+    <row r="132" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A132" s="74" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B132" s="72"/>
+      <c r="C132" s="72"/>
+      <c r="D132" s="72"/>
+      <c r="E132" s="72"/>
+    </row>
+    <row r="133" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A133" s="89" t="s">
+        <v>969</v>
+      </c>
+      <c r="B133" s="72"/>
+      <c r="C133" s="72"/>
+      <c r="D133" s="72"/>
+      <c r="E133" s="72"/>
+    </row>
+    <row r="134" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A134" s="75"/>
+      <c r="B134" s="72"/>
+      <c r="C134" s="72"/>
+      <c r="D134" s="72"/>
+      <c r="E134" s="72"/>
+    </row>
+    <row r="135" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A135" s="95" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B135" s="72"/>
+      <c r="C135" s="72"/>
+      <c r="D135" s="72"/>
+      <c r="E135" s="72"/>
+    </row>
+    <row r="136" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A136" s="95" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B136" s="72"/>
+      <c r="C136" s="72"/>
+      <c r="D136" s="72"/>
+      <c r="E136" s="72"/>
+    </row>
+    <row r="137" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A137" s="75" t="s">
+        <v>970</v>
+      </c>
+      <c r="B137" s="72"/>
+      <c r="C137" s="72"/>
+      <c r="D137" s="72"/>
+      <c r="E137" s="72"/>
+    </row>
+    <row r="138" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A138" s="96" t="s">
+        <v>778</v>
+      </c>
+      <c r="B138" s="72"/>
+      <c r="C138" s="72"/>
+      <c r="D138" s="72"/>
+      <c r="E138" s="72"/>
+    </row>
+    <row r="139" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A139" s="96" t="s">
+        <v>625</v>
+      </c>
+      <c r="B139" s="72"/>
+      <c r="C139" s="72"/>
+      <c r="D139" s="72"/>
+      <c r="E139" s="72"/>
+    </row>
+    <row r="140" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A140" s="75" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B140" s="72"/>
+      <c r="C140" s="72"/>
+      <c r="D140" s="72"/>
+      <c r="E140" s="72"/>
+    </row>
+    <row r="141" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A141" s="75" t="s">
+        <v>971</v>
+      </c>
+      <c r="B141" s="72"/>
+      <c r="C141" s="72"/>
+      <c r="D141" s="72"/>
+      <c r="E141" s="72"/>
+    </row>
+    <row r="142" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A142" s="74"/>
+      <c r="B142" s="72"/>
+      <c r="C142" s="72"/>
+      <c r="D142" s="72"/>
+      <c r="E142" s="72"/>
+    </row>
+    <row r="143" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A143" s="74" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B143" s="72"/>
+      <c r="C143" s="72"/>
+      <c r="D143" s="72"/>
+      <c r="E143" s="72"/>
+    </row>
+    <row r="144" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A144" s="89" t="s">
+        <v>972</v>
+      </c>
+      <c r="B144" s="72"/>
+      <c r="C144" s="72"/>
+      <c r="D144" s="72"/>
+      <c r="E144" s="72"/>
+    </row>
+    <row r="145" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A145" s="74" t="s">
+        <v>995</v>
+      </c>
+      <c r="B145" s="72"/>
+      <c r="C145" s="72"/>
+      <c r="D145" s="72"/>
+      <c r="E145" s="72"/>
+    </row>
+    <row r="146" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A146" s="91" t="s">
+        <v>973</v>
+      </c>
+      <c r="B146" s="92" t="s">
+        <v>974</v>
+      </c>
+      <c r="C146" s="72"/>
+      <c r="D146" s="72"/>
+      <c r="E146" s="72"/>
+    </row>
+    <row r="147" spans="1:5" s="90" customFormat="1" ht="33.75" thickBot="1">
+      <c r="A147" s="79" t="s">
+        <v>975</v>
+      </c>
+      <c r="B147" s="81" t="s">
+        <v>976</v>
+      </c>
+      <c r="C147" s="72"/>
+      <c r="D147" s="72"/>
+      <c r="E147" s="72"/>
+    </row>
+    <row r="148" spans="1:5" s="90" customFormat="1" ht="19.5">
+      <c r="A148" s="79" t="s">
+        <v>977</v>
+      </c>
+      <c r="B148" s="74" t="s">
+        <v>978</v>
+      </c>
+      <c r="C148" s="72"/>
+      <c r="D148" s="72"/>
+      <c r="E148" s="72"/>
+    </row>
+    <row r="149" spans="1:5" s="90" customFormat="1" ht="33">
+      <c r="A149" s="74" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B149" s="72"/>
+      <c r="C149" s="72"/>
+      <c r="D149" s="72"/>
+      <c r="E149" s="72"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45D8638F-2AD2-4098-8321-0BD962A63380}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetData/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update FPGA spreadsheet for PCBNo.10081
Replace the binary .xlsx workbook in PCBNo.10081/FPGA with an updated version. This is a binary change to the Excel file (no textual diff available); the spreadsheet contents were updated.
</commit_message>
<xml_diff>
--- a/PCBNo.10081/FPGA/修正履歴.xlsx
+++ b/PCBNo.10081/FPGA/修正履歴.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FPGA work\PCBNo.10081\FPGA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FPGAwork\PCBNo.10081\FPGA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F38BC98-97EE-4E89-B636-CBEA2B7A2410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9C9D21-DD22-4B18-A0AA-A38AAE8BFBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="11" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
   </bookViews>
   <sheets>
     <sheet name="修正履歴" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="1021">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="1054">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -7218,18 +7218,380 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>No1~10の確認</t>
-    <rPh sb="7" eb="9">
+    <t>No.1~10の確認</t>
+    <rPh sb="8" eb="10">
       <t>カクニン</t>
     </rPh>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>修正サマリ（6ファイル）</t>
+  </si>
+  <si>
+    <t>修正1: [致命的] FDCクロック定義のネット名修正 (MT548/MT420/MT446/MT447)</t>
+  </si>
+  <si>
+    <t>クロック定義を全削除（コメントのみに）</t>
+  </si>
+  <si>
+    <t>修正2: [中] RTLレベル syn_preserve 属性修正 (BN105/CL190/BN132)</t>
+  </si>
+  <si>
+    <t>LEDLT_TOP.vhd</t>
+  </si>
+  <si>
+    <t>slv_ctrl_top.vhd</t>
+  </si>
+  <si>
+    <t>dec6b_5b.vhd</t>
+  </si>
+  <si>
+    <t>7E, 7J, 7K, 7M の重複FDCエントリを削除</t>
+  </si>
+  <si>
+    <t>修正3: [低] encoder組合せループ警告抑制 (BN161)</t>
+  </si>
+  <si>
+    <t>encoder_2bit.vhd</t>
+  </si>
+  <si>
+    <t>全体期待効果</t>
+  </si>
+  <si>
+    <t>修正後（期待）</t>
+  </si>
+  <si>
+    <t>216件</t>
+  </si>
+  <si>
+    <t>MT548/MT420/MT529</t>
+  </si>
+  <si>
+    <t>12件</t>
+  </si>
+  <si>
+    <t>0件</t>
+  </si>
+  <si>
+    <t>BN105</t>
+  </si>
+  <si>
+    <t>27件</t>
+  </si>
+  <si>
+    <t>BN161</t>
+  </si>
+  <si>
+    <t>100件</t>
+  </si>
+  <si>
+    <t>CL190 (s_LEDPTN/s_prpty)</t>
+  </si>
+  <si>
+    <t>BN132 (DATAOUT)</t>
+  </si>
+  <si>
+    <t>6件</t>
+  </si>
+  <si>
+    <r>
+      <t>Section 0 としてクロック定義を追加。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>{n:CLKOP_t}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>{n:slv_com_top_inst.clk_gen_inst2.PLL_inst.CLKCOM_OUT}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> 等の階層パスに変更</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>期待効果</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: MT548×4、MT420×4、MT529×4、MT447×8、MT446×6 の合計 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>26件のワーニングが解消</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> され、Synplifyレベルで全PLLクロックが同一グループ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>pll_clks</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> に配置。MULTICYCLE/FALSE_PATH制約も正常に適用。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>syn_keep</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>syn_preserve</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (s_LEDPTN)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>syn_keep</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>syn_preserve</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> (s_prpty)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>syn_preserve of DATAOUT : port</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> を追加</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>期待効果</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: BN105×27件が解消。CL190のs_LEDPTN×6、s_prpty×6、BN132のDATAOUT×6 も解消見込み（合計 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>最大45件削減</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>attribute syn_loopcheck of RTL : architecture is false;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> を追加</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>期待効果</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: BN161×100件が解消見込み。FDCの </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>syn_loopcheck {0}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> もバックアップとして維持。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>~45件</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>（IPコア起因17件含む）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>次のステップ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>: Diamond 3.14で </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>Clean → Synthesize Design → 全フロー再実行</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t> してください。合成からやり直すことで、全修正がSRR/TWRに反映されます。</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="32">
+  <fonts count="37">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7458,6 +7820,36 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <name val="メイリオ"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="メイリオ"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="13.5"/>
+      <name val="メイリオ"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="メイリオ"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="メイリオ"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -7523,7 +7915,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -7814,6 +8206,45 @@
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10567,10 +10998,216 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45D8638F-2AD2-4098-8321-0BD962A63380}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A13442C-D3F5-44DA-A340-0A4C29B54C09}">
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="3" width="82.125" style="98" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="57">
+      <c r="A1" s="97" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="87">
+      <c r="A2" s="99" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="100" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="101" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="38.25" thickBot="1">
+      <c r="A4" s="102" t="s">
+        <v>693</v>
+      </c>
+      <c r="B4" s="103" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="72.75">
+      <c r="A5" s="102" t="s">
+        <v>659</v>
+      </c>
+      <c r="B5" s="104" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="131.25">
+      <c r="A6" s="105" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="65.25">
+      <c r="A7" s="99" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="100" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="101" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="19.5" thickBot="1">
+      <c r="A9" s="102" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B9" s="106" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="19.5" thickBot="1">
+      <c r="A10" s="102" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B10" s="106" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="19.5" thickBot="1">
+      <c r="A11" s="102" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B11" s="106" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="37.5">
+      <c r="A12" s="102" t="s">
+        <v>659</v>
+      </c>
+      <c r="B12" s="104" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="75">
+      <c r="A13" s="105" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="43.5">
+      <c r="A14" s="99" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="100" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="101" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="35.25">
+      <c r="A16" s="102" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B16" s="107" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="56.25">
+      <c r="A17" s="105" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="21.75">
+      <c r="A18" s="99" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="100" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="100" t="s">
+        <v>973</v>
+      </c>
+      <c r="C19" s="101" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="19.5" thickBot="1">
+      <c r="A20" s="108" t="s">
+        <v>846</v>
+      </c>
+      <c r="B20" s="108" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C20" s="109" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="19.5" thickBot="1">
+      <c r="A21" s="108" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B21" s="108" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C21" s="103" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="19.5" thickBot="1">
+      <c r="A22" s="108" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B22" s="108" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C22" s="103" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="19.5" thickBot="1">
+      <c r="A23" s="108" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B23" s="108" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C23" s="103" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="19.5" thickBot="1">
+      <c r="A24" s="108" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B24" s="108" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C24" s="103" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="108" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B25" s="108" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C25" s="104" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="93.75">
+      <c r="A26" s="105" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>